<commit_message>
Înlocuire proiect încărcat greșit
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24931"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ASUS\Documents\UiPath\ProductScrape\Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uipath-my.sharepoint.com/personal/alexandra_veizu_uipath_com/Documents/Documents/Projects/REFrameworkNET5/StudioTemplates/REFramework/contentFiles/any/any/pt2/VisualBasic/Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D371C337-46C6-4563-90BB-0F7F3AFA7919}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="13_ncr:1_{00D541BD-CB78-4D75-8532-9AD73E8C785E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F8C54E24-BA5C-4BF9-8DAB-2778512EC11B}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="45">
   <si>
     <t>Name</t>
   </si>
@@ -159,59 +159,14 @@
     <t xml:space="preserve">The maximum number of consecutive system exceptions was reached. </t>
   </si>
   <si>
-    <t>Sites</t>
-  </si>
-  <si>
-    <t>Amazon.com|Amazon.es|Amazon.de|Emag.ro|Altex.ro|pccomponentes.com</t>
-  </si>
-  <si>
-    <t>AmazonCom_Url</t>
-  </si>
-  <si>
-    <t>https://www.amazon.com</t>
-  </si>
-  <si>
-    <t>AmazonEs_Url</t>
-  </si>
-  <si>
-    <t>AmazonDe_Url</t>
-  </si>
-  <si>
-    <t>https://www.amazon.de</t>
-  </si>
-  <si>
-    <t>https://www.amazon.es</t>
-  </si>
-  <si>
-    <t>Emag_Url</t>
-  </si>
-  <si>
-    <t>https://www.emag.ro</t>
-  </si>
-  <si>
-    <t>Altex_Url</t>
-  </si>
-  <si>
-    <t>https://altex.ro</t>
-  </si>
-  <si>
-    <t>Pccomponentes_Url</t>
-  </si>
-  <si>
-    <t>https://www.pccomponentes.com</t>
-  </si>
-  <si>
-    <t>InputProduct</t>
-  </si>
-  <si>
-    <t>Samsung Smart TV</t>
+    <t>ProcessABCQueue</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5">
+  <fonts count="4">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -235,12 +190,6 @@
       <name val="Calibri"/>
       <family val="2"/>
     </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color theme="10"/>
-      <name val="Calibri"/>
-    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -259,24 +208,21 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+  <cellXfs count="5">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="2">
-    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -293,9 +239,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2013 - 2022">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -333,7 +279,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2013 - 2022">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -439,7 +385,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2013 - 2022">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -581,7 +527,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -590,12 +536,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:Z998"/>
-  <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="14.44140625" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="43.5703125" customWidth="1"/>
-    <col min="2" max="2" width="69.7109375" customWidth="1"/>
-    <col min="3" max="3" width="81.42578125" customWidth="1"/>
-    <col min="4" max="26" width="8.7109375" customWidth="1"/>
+    <col min="1" max="1" width="43.5546875" customWidth="1"/>
+    <col min="2" max="2" width="43" customWidth="1"/>
+    <col min="3" max="3" width="81.44140625" customWidth="1"/>
+    <col min="4" max="26" width="8.6640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="14.25" customHeight="1">
@@ -636,12 +582,14 @@
       <c r="A2" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="B2" s="2"/>
+      <c r="B2" s="2" t="s">
+        <v>44</v>
+      </c>
       <c r="C2" s="2" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="3" spans="1:26" ht="45">
+    <row r="3" spans="1:26" ht="43.2">
       <c r="A3" s="2" t="s">
         <v>31</v>
       </c>
@@ -651,7 +599,7 @@
       </c>
     </row>
     <row r="4" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="5" spans="1:26" ht="30">
+    <row r="5" spans="1:26" ht="28.8">
       <c r="A5" t="s">
         <v>20</v>
       </c>
@@ -662,70 +610,14 @@
         <v>23</v>
       </c>
     </row>
-    <row r="6" spans="1:26" ht="14.25" customHeight="1">
-      <c r="A6" t="s">
-        <v>44</v>
-      </c>
-      <c r="B6" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="7" spans="1:26" ht="14.25" customHeight="1">
-      <c r="A7" t="s">
-        <v>46</v>
-      </c>
-      <c r="B7" s="5" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="8" spans="1:26" ht="14.25" customHeight="1">
-      <c r="A8" t="s">
-        <v>48</v>
-      </c>
-      <c r="B8" s="5" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="9" spans="1:26" ht="14.25" customHeight="1">
-      <c r="A9" t="s">
-        <v>49</v>
-      </c>
-      <c r="B9" s="5" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="10" spans="1:26" ht="14.25" customHeight="1">
-      <c r="A10" t="s">
-        <v>52</v>
-      </c>
-      <c r="B10" s="5" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="11" spans="1:26" ht="14.25" customHeight="1">
-      <c r="A11" t="s">
-        <v>54</v>
-      </c>
-      <c r="B11" s="5" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="12" spans="1:26" ht="14.25" customHeight="1">
-      <c r="A12" t="s">
-        <v>56</v>
-      </c>
-      <c r="B12" s="5" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="13" spans="1:26" ht="14.25" customHeight="1">
-      <c r="A13" t="s">
-        <v>58</v>
-      </c>
-      <c r="B13" t="s">
-        <v>59</v>
-      </c>
-    </row>
+    <row r="6" spans="1:26" ht="14.25" customHeight="1"/>
+    <row r="7" spans="1:26" ht="14.25" customHeight="1"/>
+    <row r="8" spans="1:26" ht="14.25" customHeight="1"/>
+    <row r="9" spans="1:26" ht="14.25" customHeight="1"/>
+    <row r="10" spans="1:26" ht="14.25" customHeight="1"/>
+    <row r="11" spans="1:26" ht="14.25" customHeight="1"/>
+    <row r="12" spans="1:26" ht="14.25" customHeight="1"/>
+    <row r="13" spans="1:26" ht="14.25" customHeight="1"/>
     <row r="14" spans="1:26" ht="14.25" customHeight="1"/>
     <row r="15" spans="1:26" ht="14.25" customHeight="1"/>
     <row r="16" spans="1:26" ht="14.25" customHeight="1"/>
@@ -1713,28 +1605,20 @@
     <row r="998" ht="14.25" customHeight="1"/>
   </sheetData>
   <phoneticPr fontId="2"/>
-  <hyperlinks>
-    <hyperlink ref="B9" r:id="rId1" xr:uid="{4673B4FD-B907-4777-9E36-D9E871430CCD}"/>
-    <hyperlink ref="B8" r:id="rId2" xr:uid="{7A0BF974-DECA-4E18-9EAB-21B4AC94A08A}"/>
-    <hyperlink ref="B7" r:id="rId3" xr:uid="{0E40F4A2-FCC5-4B38-B28B-832FFC26FF5E}"/>
-    <hyperlink ref="B12" r:id="rId4" xr:uid="{3FDD5614-870A-48D8-9CD0-150CDA064EFE}"/>
-    <hyperlink ref="B11" r:id="rId5" xr:uid="{CAE736EA-B02C-47BC-BFDB-ED233235A19E}"/>
-    <hyperlink ref="B10" r:id="rId6" xr:uid="{0A9CB259-76AC-4274-ABB7-9F114848132E}"/>
-  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId7"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:Z988"/>
-  <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="14.44140625" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="41" customWidth="1"/>
     <col min="2" max="2" width="51" customWidth="1"/>
-    <col min="3" max="3" width="75.42578125" customWidth="1"/>
-    <col min="4" max="26" width="8.7109375" customWidth="1"/>
+    <col min="3" max="3" width="75.44140625" customWidth="1"/>
+    <col min="4" max="26" width="8.6640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="14.25" customHeight="1">
@@ -1771,7 +1655,7 @@
       <c r="Y1" s="1"/>
       <c r="Z1" s="1"/>
     </row>
-    <row r="2" spans="1:26" ht="30">
+    <row r="2" spans="1:26" ht="28.8">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -1782,7 +1666,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:26" ht="45">
+    <row r="3" spans="1:26" ht="43.2">
       <c r="A3" t="s">
         <v>33</v>
       </c>
@@ -1896,7 +1780,7 @@
       </c>
     </row>
     <row r="16" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="17" spans="1:3" ht="45">
+    <row r="17" spans="1:3" ht="28.8">
       <c r="A17" t="s">
         <v>40</v>
       </c>
@@ -2887,12 +2771,12 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:Z1000"/>
-  <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="14.44140625" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="31.85546875" customWidth="1"/>
-    <col min="2" max="2" width="30.140625" customWidth="1"/>
-    <col min="3" max="3" width="60.28515625" customWidth="1"/>
-    <col min="4" max="26" width="65.42578125" customWidth="1"/>
+    <col min="1" max="1" width="31.88671875" customWidth="1"/>
+    <col min="2" max="2" width="30.109375" customWidth="1"/>
+    <col min="3" max="3" width="60.33203125" customWidth="1"/>
+    <col min="4" max="26" width="65.44140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="14.25" customHeight="1">

</xml_diff>